<commit_message>
feat: clean CSR demo flow, UOM dropdown, buyer table, demo assets
- Budget/approval: raise Linda Park's authority + cost-centre budget so no
  APPROVAL_REQUIRED/BUDGET_EXCEEDED gate fires for any buyer choice
- Remove RESTRICTED_PRODUCT and SPLIT_SHIPMENT scenarios from CSR demo data
- UOM_CONVERSION: replace round-up/down table with KIT dropdown + custom entry
- Buyer resolution: registered-buyer table, email validation, agent-named prompts
- Pricing exception: drop price-waterfall table, reword as CSR DECISION NEEDED
- UI: reduce radio-select lag via on_click, robust scroll-to-top for exceptions
- Add happy-flow and CSR-approval walkthroughs + mp4 recordings and recorder
- Regenerate master-data workbooks

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/mock-data/budget-master-data.xlsx
+++ b/mock-data/budget-master-data.xlsx
@@ -821,13 +821,13 @@
         </is>
       </c>
       <c r="E4" s="4" t="n">
-        <v>80000</v>
+        <v>300000</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>78000</v>
+        <v>100000</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>2000</v>
+        <v>200000</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
@@ -1191,11 +1191,11 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>5000</v>
+        <v>200000</v>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">

</xml_diff>